<commit_message>
[AugmenredEyePopupUI] 뉴스 UI 완성
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/RobbyDialogue.xlsx
+++ b/JsonConverter/ExcelFiles/RobbyDialogue.xlsx
@@ -16,16 +16,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
   <x:si>
-    <x:t xml:space="preserve">"원더랜더즈" 가 당신의 보안체계에 새로운 위협으로 나타났다
-킴벌리 라 발레트 기자
-그 어ᄄᅠᆫ 복잡한 보안체제든 그것을 뚫는 것에 세상에서 가장 뛰어난이가 앨리스 래빗이라고 생각하셨다면, 이 새로 나타난 집단을 보고 생각을 바꾸시게 될겁니다. 이들은 아직까지 앨리스 래빗만큼 영향력 있는 모습을 보여주지 않았지만, 최근 퀸시 총리와 관련된 문제에 대해 굉장히 큰 목표를 가지고 있는 것처럼 보입니다.
-"우리는 이미 퀸시 이메일 네트워크를 장악했고, 1월달에 데이터베이스를 날려버릴 것이다" 라고 이 단체가 생방송 중 발표했습니다.
-"얄팍한 위협이다."
-퀸시 총리는 질문을 받자 "아무것도 숨기고 있지 않으니" 이메일 기록이 유출되던 djWJejs 이 그룹의 발표가 별 위협이 되지 않는다고 말했습니다.
-"모두들 내가 저번 달에 어ᄄᅠᆫ TV를 샀는지 정도나 알게 될 겁니다."
-</x:t>
-  </x:si>
-  <x:si>
     <x:t>퀸시의 새로운 경제 조정안 발표에 따라 집단 이주가 계속되고 있다.
 킴벌리 라 벨레트 기자
 세계에서 가장 높은 수준의 인플레이션과 기본적인 식료품 부족 그리고 걷잡을 수 없는 폭력 범죄율 때문에 글리치 시티의 시민들은 더 나은 삶을 찾아 다른 나라로 떠나고 있습니다.
@@ -35,31 +25,31 @@
 퀸시는 "그 작자들이 뭘 안다고 그래" 라고 결론 내렸습니다.</x:t>
   </x:si>
   <x:si>
-    <x:t>dialogue_title_1_1_000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dialogue_detail1_1_001</x:t>
-  </x:si>
-  <x:si>
-    <x:t>집단 이주가 계속되고 있습니다....</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dialogue_title_1_1_002</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dialogue_detail1_1_000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dialogue_detail1_1_002</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dialogue_title_1_1_001</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SelectionDialogueIdList</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
+    <x:t>dialogue_talk_1_001</x:t>
+  </x:si>
+  <x:si>
+    <x:t>새롭게 나타난 위협 원더랜더즈</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SelectionNameList</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dialogue_talk_1_003</x:t>
+  </x:si>
+  <x:si>
+    <x:t>하이힐을 신은 사이보그 내년 복귀.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dialogue_talk_1_000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dialogue_talk_1_002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NextDialogueId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CharacterDataId</x:t>
   </x:si>
   <x:si>
     <x:t>하이힐을 신은 사이보그가 내년 슈퍼 실버 선더 돔으로 돌아옵니다.
@@ -71,67 +61,77 @@
 몇주 뒤 이곳 어그멘티드 아이에서 단독 인터뷰 전문이 공개됩니다. 꼭 확인하세요.</x:t>
   </x:si>
   <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
     <x:t>"포어": 떠날 거야?
 질: 널 두고 떠나진 않아.</x:t>
   </x:si>
   <x:si>
-    <x:t>질: 알마 생각은 어떨지 궁금한걸...</x:t>
-  </x:si>
-  <x:si>
     <x:t>"포어": 저 사람 행동 좀 이상한데.
 질: 아마 이 사람은 자연법칙이고 뭐고 상관없나보지.</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">"원더랜더즈" 가 당신의 보안체계에 새로운 위협으로 나타났다
+킴벌리 라 발레트 기자
+그 어떠한복잡한 보안체제든 그것을 뚫는 것에 세상에서 가장 뛰어난이가 앨리스 래빗이라고 생각하셨다면, 이 새로 나타난 집단을 보고 생각을 바꾸시게 될겁니다. 이들은 아직까지 앨리스 래빗만큼 영향력 있는 모습을 보여주지 않았지만, 최근 퀸시 총리와 관련된 문제에 대해 굉장히 큰 목표를 가지고 있는 것처럼 보입니다.
+"우리는 이미 퀸시 이메일 네트워크를 장악했고, 1월달에 데이터베이스를 날려버릴 것이다" 라고 이 단체가 생방송 중 발표했습니다.
+"얄팍한 위협이다."
+퀸시 총리는 질문을 받자 "아무것도 숨기고 있지 않으니" 이메일 기록이 유출되던 어쩌던 이 그룹의 발표가 별 위협이 되지 않는다고 말했습니다.
+"모두들 내가 저번 달에 어떤 TV를 샀는지 정도나 알게 될 겁니다."
+</x:t>
+  </x:si>
+  <x:si>
     <x:t>"포어": 그래서, 그 편지는 누구한테 온거야?
 질: 아무도 아냐.</x:t>
   </x:si>
   <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
     <x:t>TexturePath</x:t>
   </x:si>
   <x:si>
-    <x:t>Description</x:t>
+    <x:t>VoicePath</x:t>
   </x:si>
   <x:si>
     <x:t>string[]</x:t>
   </x:si>
   <x:si>
-    <x:t>VoicePath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dialogue_talk_1_000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dialogue_talk_1_001</x:t>
-  </x:si>
-  <x:si>
-    <x:t>새롭게 나타난 위협 원더랜더즈</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dialogue_talk_1_002</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SelectionNameList</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dialogue_talk_1_003</x:t>
-  </x:si>
-  <x:si>
-    <x:t>하이힐을 신은 사이보그 내년 복귀.</x:t>
+    <x:t>dialogue_detail1_1_001</x:t>
+  </x:si>
+  <x:si>
+    <x:t>질: 알마 생각은 어떨지 궁금한걸...</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dialogue_title_1_1_000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dialogue_detail1_1_002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dialogue_detail1_1_000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dialogue_title_1_1_002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SelectionDialogueIdList</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dialogue_title_1_1_001</x:t>
+  </x:si>
+  <x:si>
+    <x:t>집단 이주가 계속되고 있습니다....</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
   </x:si>
   <x:si>
     <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NextDialogueId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CharacterDataId</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1033,63 +1033,63 @@
     </x:row>
     <x:row r="2" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A2" s="1" t="s">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C3" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G3" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="D3" s="2" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="E3" s="2" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F3" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="G3" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
       <x:c r="H3" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A4" s="12" t="s">
-        <x:v>2</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B4" s="5"/>
       <x:c r="C4" s="4" t="s">
-        <x:v>4</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D4" s="4"/>
       <x:c r="G4" s="4"/>
@@ -1107,11 +1107,11 @@
     </x:row>
     <x:row r="5" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A5" s="12" t="s">
-        <x:v>8</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B5" s="5"/>
       <x:c r="C5" s="4" t="s">
-        <x:v>22</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="4"/>
       <x:c r="E5" s="4"/>
@@ -1131,11 +1131,11 @@
     </x:row>
     <x:row r="6" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A6" s="12" t="s">
-        <x:v>5</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B6" s="5"/>
       <x:c r="C6" s="4" t="s">
-        <x:v>26</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D6" s="4"/>
       <x:c r="E6" s="4"/>
@@ -1155,11 +1155,11 @@
     </x:row>
     <x:row r="7" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A7" s="12" t="s">
-        <x:v>6</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B7" s="4"/>
       <x:c r="C7" s="12" t="s">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="4"/>
       <x:c r="E7" s="4"/>
@@ -1179,11 +1179,11 @@
     </x:row>
     <x:row r="8" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A8" s="12" t="s">
-        <x:v>3</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B8" s="6"/>
       <x:c r="C8" s="13" t="s">
-        <x:v>0</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D8" s="6"/>
       <x:c r="E8" s="6"/>
@@ -1203,11 +1203,11 @@
     </x:row>
     <x:row r="9" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A9" s="12" t="s">
-        <x:v>7</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B9" s="6"/>
       <x:c r="C9" s="13" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D9" s="6"/>
       <x:c r="E9" s="6"/>
@@ -1227,7 +1227,7 @@
     </x:row>
     <x:row r="10" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A10" s="4" t="s">
-        <x:v>20</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B10" s="7"/>
       <x:c r="C10" s="14" t="s">
@@ -1251,7 +1251,7 @@
     </x:row>
     <x:row r="11" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A11" s="4" t="s">
-        <x:v>21</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B11" s="7"/>
       <x:c r="C11" s="14" t="s">
@@ -1275,11 +1275,11 @@
     </x:row>
     <x:row r="12" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A12" s="4" t="s">
-        <x:v>23</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B12" s="7"/>
       <x:c r="C12" s="7" t="s">
-        <x:v>13</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D12" s="6"/>
       <x:c r="E12" s="6"/>
@@ -1299,11 +1299,11 @@
     </x:row>
     <x:row r="13" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A13" s="4" t="s">
-        <x:v>25</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B13" s="6"/>
       <x:c r="C13" s="13" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D13" s="4"/>
       <x:c r="E13" s="4"/>

</xml_diff>